<commit_message>
activity plan upload add on leave option
</commit_message>
<xml_diff>
--- a/public/assets/SMS Activity Plan Upload Format.xlsx
+++ b/public/assets/SMS Activity Plan Upload Format.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20397"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D93317E5-3BEB-475D-96CC-1D8408AC3B1D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3BD4D31-2BDC-4390-ABE2-E9226DB530C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14505" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,6 +14,17 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -78,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>YEAR</t>
   </si>
@@ -123,6 +134,9 @@
   </si>
   <si>
     <t>Lorem, ipsum dolor sit amet consectetur adipisicing elit. Maxime, error! Ex nobis quasi amet reiciendis quo asperiores ducimus fuga nisi nihil, magni cum debitis, officiis atque? Voluptatibus iste dolores voluptatem.</t>
+  </si>
+  <si>
+    <t>ON LEAVE</t>
   </si>
 </sst>
 </file>
@@ -463,7 +477,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -474,16 +488,16 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -493,9 +507,6 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -526,8 +537,8 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
@@ -536,13 +547,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -850,8 +858,8 @@
   <dimension ref="A1:H61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" style="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.5703125" style="27" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" style="25" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" style="7" customWidth="1"/>
     <col min="4" max="4" width="11.28515625" style="7" customWidth="1"/>
     <col min="5" max="5" width="10.7109375" style="7" customWidth="1"/>
@@ -865,46 +873,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30">
-        <v>2023</v>
-      </c>
-      <c r="C1" s="31"/>
-      <c r="D1" s="32" t="str">
+      <c r="B1" s="28">
+        <v>2026</v>
+      </c>
+      <c r="C1" s="29"/>
+      <c r="D1" s="30" t="str">
         <f>_xlfn.CONCAT(B1,"-",IF(B2 &lt; 10, _xlfn.CONCAT("0", B2), B2))</f>
-        <v>2023-05</v>
-      </c>
-      <c r="E1" s="31"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="34"/>
+        <v>2026-05</v>
+      </c>
+      <c r="E1" s="29"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="32"/>
     </row>
     <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="28">
+      <c r="B2" s="26">
         <v>5</v>
       </c>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="36"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="34"/>
     </row>
     <row r="3" spans="1:7" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="B3" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="38"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="36"/>
     </row>
     <row r="4" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -930,15 +938,15 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="24">
+      <c r="A5" s="23">
         <v>2</v>
       </c>
       <c r="B5" s="8" t="str">
-        <f t="shared" ref="B5:B36" si="0">TEXT($B$2&amp;"/"&amp;A5&amp;"/"&amp;$B$1, "ddd")</f>
-        <v>Tue</v>
+        <f t="shared" ref="B5:B61" si="0">TEXT($B$2&amp;"/"&amp;A5&amp;"/"&amp;$B$1, "ddd")</f>
+        <v>Thu</v>
       </c>
       <c r="C5" s="9"/>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="24" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="9" t="s">
@@ -952,788 +960,790 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="20">
+      <c r="A6" s="19">
         <v>3</v>
       </c>
-      <c r="B6" s="11" t="str">
+      <c r="B6" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Thu</v>
+      </c>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="12"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="19">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Thu</v>
+      </c>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="12"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="19">
+        <v>3</v>
+      </c>
+      <c r="B8" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Thu</v>
+      </c>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="12"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="19">
+        <v>3</v>
+      </c>
+      <c r="B9" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Thu</v>
+      </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="12"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="19">
+        <v>3</v>
+      </c>
+      <c r="B10" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Thu</v>
+      </c>
+      <c r="C10" s="11"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="12"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="19">
+        <v>3</v>
+      </c>
+      <c r="B11" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Thu</v>
+      </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="12"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="19">
+        <v>4</v>
+      </c>
+      <c r="B12" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Sun</v>
+      </c>
+      <c r="C12" s="11"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="12"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="19">
+        <v>4</v>
+      </c>
+      <c r="B13" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Sun</v>
+      </c>
+      <c r="C13" s="11"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="12"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="19">
+        <v>4</v>
+      </c>
+      <c r="B14" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Sun</v>
+      </c>
+      <c r="C14" s="11"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="12"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="19">
+        <v>4</v>
+      </c>
+      <c r="B15" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Sun</v>
+      </c>
+      <c r="C15" s="11"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="12"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="19">
+        <v>5</v>
+      </c>
+      <c r="B16" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Tue</v>
+      </c>
+      <c r="C16" s="11"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="12"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="19">
+        <v>5</v>
+      </c>
+      <c r="B17" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Tue</v>
+      </c>
+      <c r="C17" s="11"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="12"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="19">
+        <v>5</v>
+      </c>
+      <c r="B18" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Tue</v>
+      </c>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="12"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="19">
+        <v>5</v>
+      </c>
+      <c r="B19" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Tue</v>
+      </c>
+      <c r="C19" s="11"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="12"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="19">
+        <v>5</v>
+      </c>
+      <c r="B20" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Tue</v>
+      </c>
+      <c r="C20" s="11"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="12"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="19">
+        <v>8</v>
+      </c>
+      <c r="B21" s="8" t="str">
         <f t="shared" si="0"/>
         <v>Wed</v>
       </c>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="13"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="20">
-        <v>3</v>
-      </c>
-      <c r="B7" s="11" t="str">
+      <c r="C21" s="11"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="12"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="19">
+        <v>8</v>
+      </c>
+      <c r="B22" s="8" t="str">
         <f t="shared" si="0"/>
         <v>Wed</v>
       </c>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="13"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="20">
-        <v>3</v>
-      </c>
-      <c r="B8" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Wed</v>
-      </c>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="13"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="20">
-        <v>3</v>
-      </c>
-      <c r="B9" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Wed</v>
-      </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="13"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="20">
-        <v>3</v>
-      </c>
-      <c r="B10" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Wed</v>
-      </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="13"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="20">
-        <v>3</v>
-      </c>
-      <c r="B11" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Wed</v>
-      </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="13"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="20">
-        <v>4</v>
-      </c>
-      <c r="B12" s="11" t="str">
+      <c r="C22" s="11"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="12"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="19">
+        <v>9</v>
+      </c>
+      <c r="B23" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Sat</v>
+      </c>
+      <c r="C23" s="11"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="12"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="19">
+        <v>10</v>
+      </c>
+      <c r="B24" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Mon</v>
+      </c>
+      <c r="C24" s="11"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="12"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="19">
+        <v>10</v>
+      </c>
+      <c r="B25" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Mon</v>
+      </c>
+      <c r="C25" s="11"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="12"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="19">
+        <v>10</v>
+      </c>
+      <c r="B26" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Mon</v>
+      </c>
+      <c r="C26" s="11"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="12"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="19">
+        <v>10</v>
+      </c>
+      <c r="B27" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Mon</v>
+      </c>
+      <c r="C27" s="11"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="12"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="19">
+        <v>10</v>
+      </c>
+      <c r="B28" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Mon</v>
+      </c>
+      <c r="C28" s="11"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="12"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="19">
+        <v>10</v>
+      </c>
+      <c r="B29" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Mon</v>
+      </c>
+      <c r="C29" s="11"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="11"/>
+      <c r="G29" s="12"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="19">
+        <v>11</v>
+      </c>
+      <c r="B30" s="8" t="str">
         <f t="shared" si="0"/>
         <v>Thu</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="13"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="20">
-        <v>4</v>
-      </c>
-      <c r="B13" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Thu</v>
-      </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="13"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="20">
-        <v>4</v>
-      </c>
-      <c r="B14" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Thu</v>
-      </c>
-      <c r="C14" s="12"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="20">
-        <v>4</v>
-      </c>
-      <c r="B15" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Thu</v>
-      </c>
-      <c r="C15" s="12"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="13"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="20">
-        <v>5</v>
-      </c>
-      <c r="B16" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Fri</v>
-      </c>
-      <c r="C16" s="12"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="13"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="20">
-        <v>5</v>
-      </c>
-      <c r="B17" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Fri</v>
-      </c>
-      <c r="C17" s="12"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="13"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="20">
-        <v>5</v>
-      </c>
-      <c r="B18" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Fri</v>
-      </c>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="13"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="20">
-        <v>5</v>
-      </c>
-      <c r="B19" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Fri</v>
-      </c>
-      <c r="C19" s="12"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="13"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="20">
-        <v>5</v>
-      </c>
-      <c r="B20" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Fri</v>
-      </c>
-      <c r="C20" s="12"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="13"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="20">
-        <v>8</v>
-      </c>
-      <c r="B21" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Mon</v>
-      </c>
-      <c r="C21" s="12"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="13"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="20">
-        <v>8</v>
-      </c>
-      <c r="B22" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Mon</v>
-      </c>
-      <c r="C22" s="12"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="13"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="20">
-        <v>9</v>
-      </c>
-      <c r="B23" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Tue</v>
-      </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="13"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="20">
-        <v>10</v>
-      </c>
-      <c r="B24" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Wed</v>
-      </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-      <c r="G24" s="13"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="20">
-        <v>10</v>
-      </c>
-      <c r="B25" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Wed</v>
-      </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="13"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="20">
-        <v>10</v>
-      </c>
-      <c r="B26" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Wed</v>
-      </c>
-      <c r="C26" s="12"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="13"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="20">
-        <v>10</v>
-      </c>
-      <c r="B27" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Wed</v>
-      </c>
-      <c r="C27" s="12"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="13"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="20">
-        <v>10</v>
-      </c>
-      <c r="B28" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Wed</v>
-      </c>
-      <c r="C28" s="12"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="13"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="20">
-        <v>10</v>
-      </c>
-      <c r="B29" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Wed</v>
-      </c>
-      <c r="C29" s="12"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="13"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="20">
-        <v>11</v>
-      </c>
-      <c r="B30" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Thu</v>
-      </c>
-      <c r="C30" s="12"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="13"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="12"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="20">
+      <c r="A31" s="19">
         <v>12</v>
       </c>
-      <c r="B31" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Fri</v>
-      </c>
-      <c r="C31" s="12"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="13"/>
+      <c r="B31" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Sat</v>
+      </c>
+      <c r="C31" s="11"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="12"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="20">
+      <c r="A32" s="19">
         <v>15</v>
       </c>
-      <c r="B32" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Mon</v>
-      </c>
-      <c r="C32" s="12"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="12"/>
-      <c r="G32" s="13"/>
+      <c r="B32" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/15/2026</v>
+      </c>
+      <c r="C32" s="11"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="11"/>
+      <c r="G32" s="12"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="20">
+      <c r="A33" s="19">
         <v>16</v>
       </c>
-      <c r="B33" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Tue</v>
-      </c>
-      <c r="C33" s="12"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="13"/>
+      <c r="B33" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/16/2026</v>
+      </c>
+      <c r="C33" s="11"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="11"/>
+      <c r="G33" s="12"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="20">
+      <c r="A34" s="19">
         <v>16</v>
       </c>
-      <c r="B34" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Tue</v>
-      </c>
-      <c r="C34" s="12"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="13"/>
+      <c r="B34" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/16/2026</v>
+      </c>
+      <c r="C34" s="11"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="12"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="20">
+      <c r="A35" s="19">
         <v>16</v>
       </c>
-      <c r="B35" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Tue</v>
-      </c>
-      <c r="C35" s="12"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="12"/>
-      <c r="F35" s="12"/>
-      <c r="G35" s="13"/>
+      <c r="B35" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/16/2026</v>
+      </c>
+      <c r="C35" s="11"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="11"/>
+      <c r="G35" s="12"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="20">
+      <c r="A36" s="19">
         <v>16</v>
       </c>
-      <c r="B36" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>Tue</v>
-      </c>
-      <c r="C36" s="12"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
-      <c r="G36" s="13"/>
+      <c r="B36" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/16/2026</v>
+      </c>
+      <c r="C36" s="11"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
+      <c r="G36" s="12"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="20">
+      <c r="A37" s="19">
         <v>16</v>
       </c>
-      <c r="B37" s="11" t="str">
-        <f t="shared" ref="B37:B68" si="1">TEXT($B$2&amp;"/"&amp;A37&amp;"/"&amp;$B$1, "ddd")</f>
-        <v>Tue</v>
-      </c>
-      <c r="C37" s="12"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="12"/>
-      <c r="F37" s="12"/>
-      <c r="G37" s="13"/>
+      <c r="B37" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/16/2026</v>
+      </c>
+      <c r="C37" s="11"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="11"/>
+      <c r="G37" s="12"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="20">
+      <c r="A38" s="19">
         <v>16</v>
       </c>
-      <c r="B38" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Tue</v>
-      </c>
-      <c r="C38" s="12"/>
-      <c r="D38" s="16"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
-      <c r="G38" s="13"/>
+      <c r="B38" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/16/2026</v>
+      </c>
+      <c r="C38" s="11"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="11"/>
+      <c r="F38" s="11"/>
+      <c r="G38" s="12"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="20">
+      <c r="A39" s="19">
         <v>17</v>
       </c>
-      <c r="B39" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Wed</v>
-      </c>
-      <c r="C39" s="12"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="12"/>
-      <c r="F39" s="12"/>
-      <c r="G39" s="13"/>
+      <c r="B39" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/17/2026</v>
+      </c>
+      <c r="C39" s="11"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="11"/>
+      <c r="F39" s="11"/>
+      <c r="G39" s="12"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="20">
+      <c r="A40" s="19">
         <v>17</v>
       </c>
-      <c r="B40" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Wed</v>
-      </c>
-      <c r="C40" s="12"/>
-      <c r="D40" s="16"/>
-      <c r="E40" s="12"/>
-      <c r="F40" s="12"/>
-      <c r="G40" s="13"/>
+      <c r="B40" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/17/2026</v>
+      </c>
+      <c r="C40" s="11"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="11"/>
+      <c r="G40" s="12"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="20">
+      <c r="A41" s="19">
         <v>17</v>
       </c>
-      <c r="B41" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Wed</v>
-      </c>
-      <c r="C41" s="12"/>
-      <c r="D41" s="16"/>
-      <c r="E41" s="12"/>
-      <c r="F41" s="12"/>
-      <c r="G41" s="13"/>
+      <c r="B41" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/17/2026</v>
+      </c>
+      <c r="C41" s="11"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="11"/>
+      <c r="F41" s="11"/>
+      <c r="G41" s="12"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="20">
+      <c r="A42" s="19">
         <v>18</v>
       </c>
-      <c r="B42" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Thu</v>
-      </c>
-      <c r="C42" s="12"/>
-      <c r="D42" s="16"/>
-      <c r="E42" s="12"/>
-      <c r="F42" s="12"/>
-      <c r="G42" s="13"/>
+      <c r="B42" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/18/2026</v>
+      </c>
+      <c r="C42" s="11"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="11"/>
+      <c r="G42" s="12"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="20">
+      <c r="A43" s="19">
         <v>18</v>
       </c>
-      <c r="B43" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Thu</v>
-      </c>
-      <c r="C43" s="12"/>
-      <c r="D43" s="16"/>
-      <c r="E43" s="12"/>
-      <c r="F43" s="12"/>
-      <c r="G43" s="13"/>
+      <c r="B43" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/18/2026</v>
+      </c>
+      <c r="C43" s="11"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="11"/>
+      <c r="F43" s="11"/>
+      <c r="G43" s="12"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="20">
+      <c r="A44" s="19">
         <v>18</v>
       </c>
-      <c r="B44" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Thu</v>
-      </c>
-      <c r="C44" s="12"/>
-      <c r="D44" s="16"/>
-      <c r="E44" s="12"/>
-      <c r="F44" s="12"/>
-      <c r="G44" s="13"/>
+      <c r="B44" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/18/2026</v>
+      </c>
+      <c r="C44" s="11"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="11"/>
+      <c r="G44" s="12"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="20">
+      <c r="A45" s="19">
         <v>18</v>
       </c>
-      <c r="B45" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Thu</v>
-      </c>
-      <c r="C45" s="12"/>
-      <c r="D45" s="16"/>
-      <c r="E45" s="12"/>
-      <c r="F45" s="12"/>
-      <c r="G45" s="13"/>
+      <c r="B45" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/18/2026</v>
+      </c>
+      <c r="C45" s="11"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="11"/>
+      <c r="G45" s="12"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="20">
+      <c r="A46" s="19">
         <v>19</v>
       </c>
-      <c r="B46" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Fri</v>
-      </c>
-      <c r="C46" s="12"/>
-      <c r="D46" s="16"/>
-      <c r="E46" s="12"/>
-      <c r="F46" s="12"/>
-      <c r="G46" s="13"/>
+      <c r="B46" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/19/2026</v>
+      </c>
+      <c r="C46" s="11"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="11"/>
+      <c r="F46" s="11"/>
+      <c r="G46" s="12"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="20">
+      <c r="A47" s="19">
         <v>19</v>
       </c>
-      <c r="B47" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Fri</v>
-      </c>
-      <c r="C47" s="12"/>
-      <c r="D47" s="16"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="12"/>
-      <c r="G47" s="13"/>
+      <c r="B47" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/19/2026</v>
+      </c>
+      <c r="C47" s="11"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="11"/>
+      <c r="G47" s="12"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="20">
+      <c r="A48" s="19">
         <v>19</v>
       </c>
-      <c r="B48" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Fri</v>
-      </c>
-      <c r="C48" s="12"/>
-      <c r="D48" s="16"/>
-      <c r="E48" s="12"/>
-      <c r="F48" s="12"/>
-      <c r="G48" s="13"/>
+      <c r="B48" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/19/2026</v>
+      </c>
+      <c r="C48" s="11"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="11"/>
+      <c r="G48" s="12"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="20">
+      <c r="A49" s="19">
         <v>22</v>
       </c>
-      <c r="B49" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Mon</v>
-      </c>
-      <c r="C49" s="12"/>
-      <c r="D49" s="15"/>
-      <c r="E49" s="12"/>
-      <c r="F49" s="12"/>
-      <c r="G49" s="13"/>
+      <c r="B49" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/22/2026</v>
+      </c>
+      <c r="C49" s="11"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="11"/>
+      <c r="F49" s="11"/>
+      <c r="G49" s="12"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="20">
+      <c r="A50" s="19">
         <v>22</v>
       </c>
-      <c r="B50" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Mon</v>
-      </c>
-      <c r="C50" s="12"/>
-      <c r="D50" s="16"/>
-      <c r="E50" s="12"/>
-      <c r="F50" s="12"/>
-      <c r="G50" s="13"/>
+      <c r="B50" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/22/2026</v>
+      </c>
+      <c r="C50" s="11"/>
+      <c r="D50" s="15"/>
+      <c r="E50" s="11"/>
+      <c r="F50" s="11"/>
+      <c r="G50" s="12"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="20">
+      <c r="A51" s="19">
         <v>22</v>
       </c>
-      <c r="B51" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Mon</v>
-      </c>
-      <c r="C51" s="12"/>
-      <c r="D51" s="16"/>
-      <c r="E51" s="12"/>
-      <c r="F51" s="12"/>
-      <c r="G51" s="13"/>
+      <c r="B51" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/22/2026</v>
+      </c>
+      <c r="C51" s="11"/>
+      <c r="D51" s="15"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="11"/>
+      <c r="G51" s="12"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="20">
+      <c r="A52" s="19">
         <v>22</v>
       </c>
-      <c r="B52" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Mon</v>
-      </c>
-      <c r="C52" s="12"/>
-      <c r="D52" s="16"/>
-      <c r="E52" s="12"/>
-      <c r="F52" s="12"/>
-      <c r="G52" s="13"/>
+      <c r="B52" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/22/2026</v>
+      </c>
+      <c r="C52" s="11"/>
+      <c r="D52" s="15"/>
+      <c r="E52" s="11"/>
+      <c r="F52" s="11"/>
+      <c r="G52" s="12"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="20">
+      <c r="A53" s="19">
         <v>23</v>
       </c>
-      <c r="B53" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Tue</v>
-      </c>
-      <c r="C53" s="12"/>
-      <c r="D53" s="15"/>
-      <c r="E53" s="12"/>
-      <c r="F53" s="12"/>
-      <c r="G53" s="13"/>
+      <c r="B53" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/23/2026</v>
+      </c>
+      <c r="C53" s="11"/>
+      <c r="D53" s="14"/>
+      <c r="E53" s="11"/>
+      <c r="F53" s="11"/>
+      <c r="G53" s="12"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="20">
+      <c r="A54" s="19">
         <v>24</v>
       </c>
-      <c r="B54" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Wed</v>
-      </c>
-      <c r="C54" s="12"/>
-      <c r="D54" s="15"/>
-      <c r="E54" s="12"/>
-      <c r="F54" s="12"/>
-      <c r="G54" s="13"/>
+      <c r="B54" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/24/2026</v>
+      </c>
+      <c r="C54" s="11"/>
+      <c r="D54" s="14"/>
+      <c r="E54" s="11"/>
+      <c r="F54" s="11"/>
+      <c r="G54" s="12"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="20">
+      <c r="A55" s="19">
         <v>25</v>
       </c>
-      <c r="B55" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Thu</v>
-      </c>
-      <c r="C55" s="12"/>
-      <c r="D55" s="15"/>
-      <c r="E55" s="12"/>
-      <c r="F55" s="12"/>
-      <c r="G55" s="13"/>
+      <c r="B55" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/25/2026</v>
+      </c>
+      <c r="C55" s="11"/>
+      <c r="D55" s="14"/>
+      <c r="E55" s="11"/>
+      <c r="F55" s="11"/>
+      <c r="G55" s="12"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="20">
+      <c r="A56" s="19">
         <v>26</v>
       </c>
-      <c r="B56" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Fri</v>
-      </c>
-      <c r="C56" s="12"/>
-      <c r="D56" s="12"/>
-      <c r="E56" s="12"/>
-      <c r="F56" s="12"/>
-      <c r="G56" s="13"/>
+      <c r="B56" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/26/2026</v>
+      </c>
+      <c r="C56" s="11"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="11"/>
+      <c r="F56" s="11"/>
+      <c r="G56" s="12"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="20">
+      <c r="A57" s="19">
         <v>26</v>
       </c>
-      <c r="B57" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Fri</v>
-      </c>
-      <c r="C57" s="12"/>
-      <c r="D57" s="12"/>
-      <c r="E57" s="12"/>
-      <c r="F57" s="12"/>
-      <c r="G57" s="13"/>
+      <c r="B57" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/26/2026</v>
+      </c>
+      <c r="C57" s="11"/>
+      <c r="D57" s="11"/>
+      <c r="E57" s="11"/>
+      <c r="F57" s="11"/>
+      <c r="G57" s="12"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="20">
+      <c r="A58" s="19">
         <v>29</v>
       </c>
-      <c r="B58" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Mon</v>
-      </c>
-      <c r="C58" s="12"/>
-      <c r="D58" s="15"/>
-      <c r="E58" s="12"/>
-      <c r="F58" s="12"/>
-      <c r="G58" s="13"/>
+      <c r="B58" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/29/2026</v>
+      </c>
+      <c r="C58" s="11"/>
+      <c r="D58" s="14"/>
+      <c r="E58" s="11"/>
+      <c r="F58" s="11"/>
+      <c r="G58" s="12"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="20">
+      <c r="A59" s="19">
         <v>29</v>
       </c>
-      <c r="B59" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Mon</v>
-      </c>
-      <c r="C59" s="12"/>
-      <c r="D59" s="16"/>
-      <c r="E59" s="12"/>
-      <c r="F59" s="12"/>
-      <c r="G59" s="13"/>
+      <c r="B59" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/29/2026</v>
+      </c>
+      <c r="C59" s="11"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="11"/>
+      <c r="F59" s="11"/>
+      <c r="G59" s="12"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="20">
+      <c r="A60" s="19">
         <v>30</v>
       </c>
-      <c r="B60" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>Tue</v>
-      </c>
-      <c r="C60" s="12"/>
-      <c r="D60" s="15"/>
-      <c r="E60" s="12"/>
-      <c r="F60" s="12"/>
-      <c r="G60" s="13"/>
+      <c r="B60" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/30/2026</v>
+      </c>
+      <c r="C60" s="11"/>
+      <c r="D60" s="14"/>
+      <c r="E60" s="11"/>
+      <c r="F60" s="11"/>
+      <c r="G60" s="12"/>
     </row>
     <row r="61" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="21">
+      <c r="A61" s="20">
         <v>31</v>
       </c>
-      <c r="B61" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v>Wed</v>
-      </c>
-      <c r="C61" s="17"/>
-      <c r="D61" s="18"/>
-      <c r="E61" s="14"/>
-      <c r="F61" s="14"/>
-      <c r="G61" s="19"/>
+      <c r="B61" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>5/31/2026</v>
+      </c>
+      <c r="C61" s="16"/>
+      <c r="D61" s="17"/>
+      <c r="E61" s="13"/>
+      <c r="F61" s="13"/>
+      <c r="G61" s="18"/>
     </row>
   </sheetData>
   <dataConsolidate/>

</xml_diff>